<commit_message>
altri fix agli orari
</commit_message>
<xml_diff>
--- a/ORARI CLASSI/input_excel/Orario_per_Aule_Completo.xlsx
+++ b/ORARI CLASSI/input_excel/Orario_per_Aule_Completo.xlsx
@@ -814,7 +814,7 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>* BASI DI DATI (A-H)</t>
+          <t>BASI DI DATI (A-H)</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -985,7 +985,7 @@
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>* BASI DI DATI (A-H)</t>
+          <t>BASI DI DATI (A-H)</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
@@ -1184,7 +1184,7 @@
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>* BASI DI DATI (A-H)</t>
+          <t>BASI DI DATI (A-H)</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
@@ -1308,7 +1308,11 @@
           <t>CYBERSECURITY FOR HEALTHCARE</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>IDROLOGIA</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr">
         <is>
           <t>COSTRUZIONE DI MACCHINE ED ELEMENTI FINITI</t>
@@ -1461,11 +1465,7 @@
           <t>INDUSTRIAL MICROBIOLOGY - MICROBIOLOGIA INDUSTRIALE</t>
         </is>
       </c>
-      <c r="AX5" t="inlineStr">
-        <is>
-          <t>IDROLOGIA</t>
-        </is>
-      </c>
+      <c r="AX5" t="inlineStr"/>
       <c r="AY5" t="inlineStr"/>
       <c r="AZ5" t="inlineStr"/>
       <c r="BA5" t="inlineStr"/>
@@ -1507,7 +1507,11 @@
           <t>SYSTEM ON CHIP</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>IDROLOGIA</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr">
         <is>
@@ -1620,11 +1624,7 @@
       <c r="AU6" t="inlineStr"/>
       <c r="AV6" t="inlineStr"/>
       <c r="AW6" t="inlineStr"/>
-      <c r="AX6" t="inlineStr">
-        <is>
-          <t>IDROLOGIA</t>
-        </is>
-      </c>
+      <c r="AX6" t="inlineStr"/>
       <c r="AY6" t="inlineStr"/>
       <c r="AZ6" t="inlineStr"/>
       <c r="BA6" t="inlineStr"/>
@@ -1806,7 +1806,11 @@
           <t>ECOLOGIA INDUSTRIALE</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>SISTEMI DI MISURA PER L'INDUSTRIA 4.0</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr">
         <is>
           <t>MODELLISTICA DEI SISTEMI ENERGETICI E PROPULSIVI</t>
@@ -1948,11 +1952,7 @@
       </c>
       <c r="AX8" t="inlineStr"/>
       <c r="AY8" t="inlineStr"/>
-      <c r="AZ8" t="inlineStr">
-        <is>
-          <t>SISTEMI DI MISURA PER L'INDUSTRIA 4.0</t>
-        </is>
-      </c>
+      <c r="AZ8" t="inlineStr"/>
       <c r="BA8" t="inlineStr"/>
       <c r="BB8" t="inlineStr"/>
       <c r="BC8" t="inlineStr">
@@ -1989,7 +1989,11 @@
           <t>ECOLOGIA INDUSTRIALE</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>SISTEMI DI MISURA PER L'INDUSTRIA 4.0</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr">
         <is>
           <t>MODELLISTICA DEI SISTEMI ENERGETICI E PROPULSIVI</t>
@@ -1997,7 +2001,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>* CLOUD SYSTEMS AND ADVANCED NETWORKING</t>
+          <t>CLOUD SYSTEMS AND ADVANCED NETWORKING</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -2071,7 +2075,7 @@
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>* BASI DI DATI (I-Z)</t>
+          <t>BASI DI DATI (I-Z)</t>
         </is>
       </c>
       <c r="AA9" t="inlineStr"/>
@@ -2143,11 +2147,7 @@
           <t>OPERATIONS AND MAINTENANCE MANAGEMENT IN SMART MANUFACTURING SYSTEMS</t>
         </is>
       </c>
-      <c r="AZ9" t="inlineStr">
-        <is>
-          <t>SISTEMI DI MISURA PER L'INDUSTRIA 4.0</t>
-        </is>
-      </c>
+      <c r="AZ9" t="inlineStr"/>
       <c r="BA9" t="inlineStr"/>
       <c r="BB9" t="inlineStr"/>
       <c r="BC9" t="inlineStr">
@@ -2184,7 +2184,11 @@
           <t>PROCESSI SOSTENIBILI DELLA CHIMICA INDUSTRIALE</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>SISTEMI DI MISURA PER L'INDUSTRIA 4.0</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
           <t>TECHNOLOGIES AND METHODS FOR ENERGY MANAGEMENT IN SMART INDUSTRIES</t>
@@ -2192,7 +2196,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>* CLOUD SYSTEMS AND ADVANCED NETWORKING</t>
+          <t>CLOUD SYSTEMS AND ADVANCED NETWORKING</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -2262,7 +2266,7 @@
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>* BASI DI DATI (I-Z)</t>
+          <t>BASI DI DATI (I-Z)</t>
         </is>
       </c>
       <c r="AA10" t="inlineStr">
@@ -2334,11 +2338,7 @@
           <t>OPERATIONS AND MAINTENANCE MANAGEMENT IN SMART MANUFACTURING SYSTEMS</t>
         </is>
       </c>
-      <c r="AZ10" t="inlineStr">
-        <is>
-          <t>SISTEMI DI MISURA PER L'INDUSTRIA 4.0</t>
-        </is>
-      </c>
+      <c r="AZ10" t="inlineStr"/>
       <c r="BA10" t="inlineStr"/>
       <c r="BB10" t="inlineStr"/>
       <c r="BC10" t="inlineStr"/>
@@ -2375,7 +2375,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>* CLOUD SYSTEMS AND ADVANCED NETWORKING</t>
+          <t>CLOUD SYSTEMS AND ADVANCED NETWORKING</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -2441,7 +2441,7 @@
       </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>* BASI DI DATI (I-Z)</t>
+          <t>BASI DI DATI (I-Z)</t>
         </is>
       </c>
       <c r="AA11" t="inlineStr">
@@ -2834,7 +2834,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>* TECNOLOGIE ELETTRICHE PER L'INFORMATICA INDUSTRIALE</t>
+          <t>TECNOLOGIE ELETTRICHE PER L'INFORMATICA INDUSTRIALE</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -2916,7 +2916,7 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>*AI</t>
+          <t>INTELLIGENZA ARTIFICIALE: METODI ED APPLICAZIONI</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -2963,7 +2963,7 @@
       <c r="AR2" t="inlineStr"/>
       <c r="AS2" t="inlineStr">
         <is>
-          <t>* ANTENNE</t>
+          <t>PROGETTAZIONE IMPIANTI DI RETE CABLATI E WIRELESS</t>
         </is>
       </c>
       <c r="AT2" t="inlineStr"/>
@@ -3021,7 +3021,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>* TECNOLOGIE ELETTRICHE PER L'INFORMATICA INDUSTRIALE</t>
+          <t>TECNOLOGIE ELETTRICHE PER L'INFORMATICA INDUSTRIALE</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -3107,7 +3107,7 @@
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>*AI</t>
+          <t>INTELLIGENZA ARTIFICIALE: METODI ED APPLICAZIONI</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
@@ -3154,7 +3154,7 @@
       <c r="AR3" t="inlineStr"/>
       <c r="AS3" t="inlineStr">
         <is>
-          <t>* ANTENNE</t>
+          <t>PROGETTAZIONE IMPIANTI DI RETE CABLATI E WIRELESS</t>
         </is>
       </c>
       <c r="AT3" t="inlineStr">
@@ -3276,7 +3276,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>* NATURAL LANGUAGE PROCESSING  AND LARGE LANGUAGE MODELS</t>
+          <t>NATURAL LANGUAGE PROCESSING  AND LARGE LANGUAGE MODELS</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -3302,7 +3302,7 @@
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>* STATISTICA APPLICATA</t>
+          <t>STATISTICA APPLICATA</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
@@ -3463,7 +3463,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>* NATURAL LANGUAGE PROCESSING  AND LARGE LANGUAGE MODELS</t>
+          <t>NATURAL LANGUAGE PROCESSING  AND LARGE LANGUAGE MODELS</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -3489,7 +3489,7 @@
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>* STATISTICA APPLICATA</t>
+          <t>STATISTICA APPLICATA</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr">
@@ -3634,7 +3634,7 @@
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr">
         <is>
-          <t>* NATURAL LANGUAGE PROCESSING  AND LARGE LANGUAGE MODELS</t>
+          <t>NATURAL LANGUAGE PROCESSING  AND LARGE LANGUAGE MODELS</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -3660,7 +3660,7 @@
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>* PROGRAMMAZIONE JAVA AVANZATA</t>
+          <t>PROGRAMMAZIONE JAVA AVANZATA</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
@@ -3769,7 +3769,7 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>* INTELLIGENT ROBOT NAVIGATION</t>
+          <t>INTELLIGENT ROBOT NAVIGATION</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -3835,7 +3835,7 @@
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>* PROGRAMMAZIONE JAVA AVANZATA</t>
+          <t>PROGRAMMAZIONE JAVA AVANZATA</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr"/>
@@ -3944,7 +3944,7 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>* INTELLIGENT ROBOT NAVIGATION</t>
+          <t>INTELLIGENT ROBOT NAVIGATION</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -4022,7 +4022,7 @@
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>* PROGRAMMAZIONE JAVA AVANZATA</t>
+          <t>PROGRAMMAZIONE JAVA AVANZATA</t>
         </is>
       </c>
       <c r="AA8" t="inlineStr">
@@ -4217,7 +4217,7 @@
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AI APPLICATIONS</t>
         </is>
       </c>
       <c r="AA9" t="inlineStr">
@@ -4256,7 +4256,7 @@
       <c r="AN9" t="inlineStr"/>
       <c r="AO9" t="inlineStr">
         <is>
-          <t>* CYBERSECURITY APPLICATIONS</t>
+          <t>CYBERSECURITY</t>
         </is>
       </c>
       <c r="AP9" t="inlineStr">
@@ -4420,7 +4420,7 @@
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AI APPLICATIONS</t>
         </is>
       </c>
       <c r="AA10" t="inlineStr">
@@ -4455,7 +4455,7 @@
       <c r="AN10" t="inlineStr"/>
       <c r="AO10" t="inlineStr">
         <is>
-          <t>* CYBERSECURITY APPLICATIONS</t>
+          <t>CYBERSECURITY</t>
         </is>
       </c>
       <c r="AP10" t="inlineStr">
@@ -4988,7 +4988,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>* CLOUD SYSTEMS AND ADVANCED NETWORKING</t>
+          <t>CLOUD SYSTEMS AND ADVANCED NETWORKING</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -5066,7 +5066,7 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>* BASI DI DATI (I-Z)</t>
+          <t>BASI DI DATI (I-Z)</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -5175,7 +5175,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>* CLOUD SYSTEMS AND ADVANCED NETWORKING</t>
+          <t>CLOUD SYSTEMS AND ADVANCED NETWORKING</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -5257,7 +5257,7 @@
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>* BASI DI DATI (I-Z)</t>
+          <t>BASI DI DATI (I-Z)</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
@@ -5766,11 +5766,7 @@
       </c>
       <c r="BA5" t="inlineStr"/>
       <c r="BB5" t="inlineStr"/>
-      <c r="BC5" t="inlineStr">
-        <is>
-          <t>LABORATORIO DI ORGANIZZAZIONE E SICUREZZA DEI CANTIERI EDILI E DELLE INFRASTRUTTURE</t>
-        </is>
-      </c>
+      <c r="BC5" t="inlineStr"/>
       <c r="BD5" t="inlineStr"/>
       <c r="BE5" t="inlineStr"/>
     </row>
@@ -5953,11 +5949,7 @@
       <c r="AZ6" t="inlineStr"/>
       <c r="BA6" t="inlineStr"/>
       <c r="BB6" t="inlineStr"/>
-      <c r="BC6" t="inlineStr">
-        <is>
-          <t>LABORATORIO DI ORGANIZZAZIONE E SICUREZZA DEI CANTIERI EDILI E DELLE INFRASTRUTTURE</t>
-        </is>
-      </c>
+      <c r="BC6" t="inlineStr"/>
       <c r="BD6" t="inlineStr"/>
       <c r="BE6" t="inlineStr"/>
     </row>
@@ -6132,11 +6124,7 @@
       <c r="AZ7" t="inlineStr"/>
       <c r="BA7" t="inlineStr"/>
       <c r="BB7" t="inlineStr"/>
-      <c r="BC7" t="inlineStr">
-        <is>
-          <t>LABORATORIO DI ORGANIZZAZIONE E SICUREZZA DEI CANTIERI EDILI E DELLE INFRASTRUTTURE</t>
-        </is>
-      </c>
+      <c r="BC7" t="inlineStr"/>
       <c r="BD7" t="inlineStr"/>
       <c r="BE7" t="inlineStr"/>
     </row>
@@ -6374,7 +6362,11 @@
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>LABORATORIO DI ORGANIZZAZIONE E SICUREZZA DEI CANTIERI EDILI E DELLE INFRASTRUTTURE</t>
+        </is>
+      </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>FISICA II</t>
@@ -6557,7 +6549,11 @@
           <t>LEAN OPERATIONS MANAGEMENT</t>
         </is>
       </c>
-      <c r="K10" t="inlineStr"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>LABORATORIO DI ORGANIZZAZIONE E SICUREZZA DEI CANTIERI EDILI E DELLE INFRASTRUTTURE</t>
+        </is>
+      </c>
       <c r="L10" t="inlineStr">
         <is>
           <t>FONDAMENTI DI INFORMATICA E BASI DI DATI</t>
@@ -6622,7 +6618,7 @@
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>* BASI DI DATI (A-H)</t>
+          <t>BASI DI DATI (A-H)</t>
         </is>
       </c>
       <c r="AA10" t="inlineStr">
@@ -6682,11 +6678,7 @@
           <t>IMPIANTI ELETTRICI AD USO CIVILE</t>
         </is>
       </c>
-      <c r="AZ10" t="inlineStr">
-        <is>
-          <t>ELECTRIC MACHINES AND DRIVES FOR SMART INDUSTRY</t>
-        </is>
-      </c>
+      <c r="AZ10" t="inlineStr"/>
       <c r="BA10" t="inlineStr">
         <is>
           <t>FONDAMENTI DI MISURE E STRUMENTAZIONE VIRTUALE</t>
@@ -6740,7 +6732,11 @@
           <t>LEAN OPERATIONS MANAGEMENT</t>
         </is>
       </c>
-      <c r="K11" t="inlineStr"/>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>LABORATORIO DI ORGANIZZAZIONE E SICUREZZA DEI CANTIERI EDILI E DELLE INFRASTRUTTURE</t>
+        </is>
+      </c>
       <c r="L11" t="inlineStr">
         <is>
           <t>FONDAMENTI DI INFORMATICA E BASI DI DATI</t>
@@ -6805,7 +6801,7 @@
       </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>* BASI DI DATI (A-H)</t>
+          <t>BASI DI DATI (A-H)</t>
         </is>
       </c>
       <c r="AA11" t="inlineStr">
@@ -6853,11 +6849,7 @@
       </c>
       <c r="AX11" t="inlineStr"/>
       <c r="AY11" t="inlineStr"/>
-      <c r="AZ11" t="inlineStr">
-        <is>
-          <t>ELECTRIC MACHINES AND DRIVES FOR SMART INDUSTRY</t>
-        </is>
-      </c>
+      <c r="AZ11" t="inlineStr"/>
       <c r="BA11" t="inlineStr">
         <is>
           <t>FONDAMENTI DI MISURE E STRUMENTAZIONE VIRTUALE</t>
@@ -7202,7 +7194,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>* ANTENNE</t>
+          <t>PROGETTAZIONE IMPIANTI DI RETE CABLATI E WIRELESS</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
@@ -7280,7 +7272,7 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>*AI</t>
+          <t>INTELLIGENZA ARTIFICIALE: METODI ED APPLICAZIONI</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -7319,7 +7311,7 @@
       <c r="AN2" t="inlineStr"/>
       <c r="AO2" t="inlineStr">
         <is>
-          <t>* TECNOLOGIE ELETTRICHE PER L'INFORMATICA INDUSTRIALE</t>
+          <t>TECNOLOGIE ELETTRICHE PER L'INFORMATICA INDUSTRIALE</t>
         </is>
       </c>
       <c r="AP2" t="inlineStr"/>
@@ -7381,7 +7373,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>* ANTENNE</t>
+          <t>PROGETTAZIONE IMPIANTI DI RETE CABLATI E WIRELESS</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -7463,7 +7455,7 @@
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>*AI</t>
+          <t>INTELLIGENZA ARTIFICIALE: METODI ED APPLICAZIONI</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
@@ -7502,7 +7494,7 @@
       <c r="AN3" t="inlineStr"/>
       <c r="AO3" t="inlineStr">
         <is>
-          <t>* TECNOLOGIE ELETTRICHE PER L'INFORMATICA INDUSTRIALE</t>
+          <t>TECNOLOGIE ELETTRICHE PER L'INFORMATICA INDUSTRIALE</t>
         </is>
       </c>
       <c r="AP3" t="inlineStr"/>
@@ -7576,7 +7568,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>* ANTENNE</t>
+          <t>PROGETTAZIONE IMPIANTI DI RETE CABLATI E WIRELESS</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -7658,7 +7650,7 @@
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>*AI</t>
+          <t>INTELLIGENZA ARTIFICIALE: METODI ED APPLICAZIONI</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
@@ -7705,7 +7697,7 @@
       <c r="AN4" t="inlineStr"/>
       <c r="AO4" t="inlineStr">
         <is>
-          <t>* TECNOLOGIE ELETTRICHE PER L'INFORMATICA INDUSTRIALE</t>
+          <t>TECNOLOGIE ELETTRICHE PER L'INFORMATICA INDUSTRIALE</t>
         </is>
       </c>
       <c r="AP4" t="inlineStr"/>
@@ -7791,7 +7783,11 @@
           <t>SOSTENIBILITÀ ENERGETICA ED AMBIENTALE</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>GESTIONE DEGLI IMPIANTI DI PROCESSO</t>
+        </is>
+      </c>
       <c r="K5" t="inlineStr">
         <is>
           <t>ADVANCED COMPUTATIONAL MECHANICS WITH APPLICATIONS TO COMPOSITE MATERIALS AND STRUCTURES</t>
@@ -7835,7 +7831,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>* NATURAL LANGUAGE PROCESSING  AND LARGE LANGUAGE MODELS</t>
+          <t>NATURAL LANGUAGE PROCESSING  AND LARGE LANGUAGE MODELS</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -7865,7 +7861,7 @@
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>* CYBERSECURITY APPLICATIONS</t>
+          <t>CYBERSECURITY</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr">
@@ -7920,7 +7916,7 @@
       <c r="AR5" t="inlineStr"/>
       <c r="AS5" t="inlineStr">
         <is>
-          <t>* IOT APPLICATIONS</t>
+          <t>MOBILE PROGRAMMING</t>
         </is>
       </c>
       <c r="AT5" t="inlineStr">
@@ -8002,7 +7998,11 @@
           <t>SOSTENIBILITÀ ENERGETICA ED AMBIENTALE</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>GESTIONE DEGLI IMPIANTI DI PROCESSO</t>
+        </is>
+      </c>
       <c r="K6" t="inlineStr">
         <is>
           <t>ADVANCED COMPUTATIONAL MECHANICS WITH APPLICATIONS TO COMPOSITE MATERIALS AND STRUCTURES</t>
@@ -8046,7 +8046,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>* NATURAL LANGUAGE PROCESSING  AND LARGE LANGUAGE MODELS</t>
+          <t>NATURAL LANGUAGE PROCESSING  AND LARGE LANGUAGE MODELS</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -8072,7 +8072,7 @@
       </c>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>* CYBERSECURITY APPLICATIONS</t>
+          <t>CYBERSECURITY</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
@@ -8115,7 +8115,7 @@
       <c r="AR6" t="inlineStr"/>
       <c r="AS6" t="inlineStr">
         <is>
-          <t>* IOT APPLICATIONS</t>
+          <t>MOBILE PROGRAMMING</t>
         </is>
       </c>
       <c r="AT6" t="inlineStr">
@@ -8235,7 +8235,7 @@
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AI APPLICATIONS</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr">
@@ -8274,7 +8274,7 @@
       <c r="AN7" t="inlineStr"/>
       <c r="AO7" t="inlineStr">
         <is>
-          <t>DIGITAL MEDICINE APPLICATIONS</t>
+          <t>MEDICAL WEARABLE DEVICES</t>
         </is>
       </c>
       <c r="AP7" t="inlineStr"/>
@@ -8310,11 +8310,7 @@
       </c>
       <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>GESTIONE DEGLI IMPIANTI DI PROCESSO</t>
-        </is>
-      </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>COMBUSTIONE</t>
@@ -8418,7 +8414,7 @@
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>nan</t>
+          <t>AI APPLICATIONS</t>
         </is>
       </c>
       <c r="AA8" t="inlineStr">
@@ -8453,7 +8449,7 @@
       <c r="AN8" t="inlineStr"/>
       <c r="AO8" t="inlineStr">
         <is>
-          <t>DIGITAL MEDICINE APPLICATIONS</t>
+          <t>MEDICAL WEARABLE DEVICES</t>
         </is>
       </c>
       <c r="AP8" t="inlineStr"/>
@@ -8509,11 +8505,7 @@
           <t>TRASPORTO MERCI E LOGISTICA</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>GESTIONE DEGLI IMPIANTI DI PROCESSO</t>
-        </is>
-      </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>COMBUSTIONE</t>
@@ -8531,7 +8523,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>* INTELLIGENT ROBOT NAVIGATION</t>
+          <t>INTELLIGENT ROBOT NAVIGATION</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -8609,7 +8601,7 @@
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>* STATISTICA APPLICATA</t>
+          <t>STATISTICA APPLICATA</t>
         </is>
       </c>
       <c r="AA9" t="inlineStr">
@@ -8669,11 +8661,7 @@
       </c>
       <c r="AX9" t="inlineStr"/>
       <c r="AY9" t="inlineStr"/>
-      <c r="AZ9" t="inlineStr">
-        <is>
-          <t>ELECTRIC MACHINES AND DRIVES FOR SMART INDUSTRY</t>
-        </is>
-      </c>
+      <c r="AZ9" t="inlineStr"/>
       <c r="BA9" t="inlineStr"/>
       <c r="BB9" t="inlineStr"/>
       <c r="BC9" t="inlineStr">
@@ -8714,7 +8702,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>* INTELLIGENT ROBOT NAVIGATION</t>
+          <t>INTELLIGENT ROBOT NAVIGATION</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -8792,7 +8780,7 @@
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>* STATISTICA APPLICATA</t>
+          <t>STATISTICA APPLICATA</t>
         </is>
       </c>
       <c r="AA10" t="inlineStr">
@@ -8864,11 +8852,7 @@
           <t>ANALISI E MITIGAZIONE DEL RISCHIO DA FRANA</t>
         </is>
       </c>
-      <c r="AZ10" t="inlineStr">
-        <is>
-          <t>ELECTRIC MACHINES AND DRIVES FOR SMART INDUSTRY</t>
-        </is>
-      </c>
+      <c r="AZ10" t="inlineStr"/>
       <c r="BA10" t="inlineStr"/>
       <c r="BB10" t="inlineStr"/>
       <c r="BC10" t="inlineStr"/>
@@ -8901,7 +8885,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>* INTELLIGENT ROBOT NAVIGATION</t>
+          <t>INTELLIGENT ROBOT NAVIGATION</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -8975,7 +8959,7 @@
       </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>* STATISTICA APPLICATA</t>
+          <t>STATISTICA APPLICATA</t>
         </is>
       </c>
       <c r="AA11" t="inlineStr">
@@ -9035,11 +9019,7 @@
           <t>ANALISI E MITIGAZIONE DEL RISCHIO DA FRANA</t>
         </is>
       </c>
-      <c r="AZ11" t="inlineStr">
-        <is>
-          <t>ELECTRIC MACHINES AND DRIVES FOR SMART INDUSTRY</t>
-        </is>
-      </c>
+      <c r="AZ11" t="inlineStr"/>
       <c r="BA11" t="inlineStr"/>
       <c r="BB11" t="inlineStr"/>
       <c r="BC11" t="inlineStr"/>
@@ -9450,7 +9430,7 @@
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>* BASI DI DATI (A-H)</t>
+          <t>BASI DI DATI (A-H)</t>
         </is>
       </c>
       <c r="AA2" t="inlineStr">
@@ -9633,7 +9613,7 @@
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>* BASI DI DATI (A-H)</t>
+          <t>BASI DI DATI (A-H)</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
@@ -9816,7 +9796,7 @@
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>* BASI DI DATI (A-H)</t>
+          <t>BASI DI DATI (A-H)</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
@@ -9995,7 +9975,7 @@
       </c>
       <c r="Z5" t="inlineStr">
         <is>
-          <t>* PROGRAMMAZIONE JAVA AVANZATA</t>
+          <t>PROGRAMMAZIONE JAVA AVANZATA</t>
         </is>
       </c>
       <c r="AA5" t="inlineStr">
@@ -10154,7 +10134,7 @@
       <c r="Y6" t="inlineStr"/>
       <c r="Z6" t="inlineStr">
         <is>
-          <t>* PROGRAMMAZIONE JAVA AVANZATA</t>
+          <t>PROGRAMMAZIONE JAVA AVANZATA</t>
         </is>
       </c>
       <c r="AA6" t="inlineStr">
@@ -10305,7 +10285,7 @@
       </c>
       <c r="Z7" t="inlineStr">
         <is>
-          <t>* IOT APPLICATIONS</t>
+          <t>MOBILE PROGRAMMING</t>
         </is>
       </c>
       <c r="AA7" t="inlineStr"/>
@@ -10330,15 +10310,15 @@
       <c r="AL7" t="inlineStr"/>
       <c r="AM7" t="inlineStr"/>
       <c r="AN7" t="inlineStr"/>
-      <c r="AO7" t="inlineStr"/>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>MEDICAL WEARABLE DEVICES</t>
+        </is>
+      </c>
       <c r="AP7" t="inlineStr"/>
       <c r="AQ7" t="inlineStr"/>
       <c r="AR7" t="inlineStr"/>
-      <c r="AS7" t="inlineStr">
-        <is>
-          <t>DIGITAL MEDICINE APPLICATIONS</t>
-        </is>
-      </c>
+      <c r="AS7" t="inlineStr"/>
       <c r="AT7" t="inlineStr"/>
       <c r="AU7" t="inlineStr"/>
       <c r="AV7" t="inlineStr"/>
@@ -10444,7 +10424,7 @@
       </c>
       <c r="Z8" t="inlineStr">
         <is>
-          <t>* IOT APPLICATIONS</t>
+          <t>MOBILE PROGRAMMING</t>
         </is>
       </c>
       <c r="AA8" t="inlineStr">
@@ -10465,7 +10445,11 @@
       <c r="AL8" t="inlineStr"/>
       <c r="AM8" t="inlineStr"/>
       <c r="AN8" t="inlineStr"/>
-      <c r="AO8" t="inlineStr"/>
+      <c r="AO8" t="inlineStr">
+        <is>
+          <t>MEDICAL WEARABLE DEVICES</t>
+        </is>
+      </c>
       <c r="AP8" t="inlineStr">
         <is>
           <t>LABORATORIO DI INFORMATICA GRAFICA E BIM</t>
@@ -10473,11 +10457,7 @@
       </c>
       <c r="AQ8" t="inlineStr"/>
       <c r="AR8" t="inlineStr"/>
-      <c r="AS8" t="inlineStr">
-        <is>
-          <t>DIGITAL MEDICINE APPLICATIONS</t>
-        </is>
-      </c>
+      <c r="AS8" t="inlineStr"/>
       <c r="AT8" t="inlineStr"/>
       <c r="AU8" t="inlineStr"/>
       <c r="AV8" t="inlineStr"/>
@@ -10587,7 +10567,7 @@
       </c>
       <c r="Z9" t="inlineStr">
         <is>
-          <t>* BASI DI DATI (I-Z)</t>
+          <t>BASI DI DATI (I-Z)</t>
         </is>
       </c>
       <c r="AA9" t="inlineStr">
@@ -10730,7 +10710,7 @@
       </c>
       <c r="Z10" t="inlineStr">
         <is>
-          <t>* BASI DI DATI (I-Z)</t>
+          <t>BASI DI DATI (I-Z)</t>
         </is>
       </c>
       <c r="AA10" t="inlineStr">
@@ -10857,7 +10837,7 @@
       </c>
       <c r="Z11" t="inlineStr">
         <is>
-          <t>* BASI DI DATI (I-Z)</t>
+          <t>BASI DI DATI (I-Z)</t>
         </is>
       </c>
       <c r="AA11" t="inlineStr"/>

</xml_diff>

<commit_message>
1^ sem. 26/27 pt.3
</commit_message>
<xml_diff>
--- a/ORARI CLASSI/input_excel/Orario_per_Aule_Completo.xlsx
+++ b/ORARI CLASSI/input_excel/Orario_per_Aule_Completo.xlsx
@@ -743,7 +743,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>CHIMICA</t>
+          <t>MATEMATICA I</t>
         </is>
       </c>
       <c r="U2" t="inlineStr"/>
@@ -772,11 +772,7 @@
           <t>FENOMENI DI TRASPORTO</t>
         </is>
       </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>RESTAURO ARCHITETTONICO</t>
-        </is>
-      </c>
+      <c r="AA2" t="inlineStr"/>
       <c r="AB2" t="inlineStr">
         <is>
           <t>ELETTROTECNICA (I-Z)</t>
@@ -813,11 +809,7 @@
           <t>PROCESS UNIT OPERATIONS - OPERAZIONI UNITARIE NELL'INDUSTRIA DI PROCESSO</t>
         </is>
       </c>
-      <c r="AR2" t="inlineStr">
-        <is>
-          <t>COMPLEMENTI DI MATEMATICA</t>
-        </is>
-      </c>
+      <c r="AR2" t="inlineStr"/>
       <c r="AS2" t="inlineStr">
         <is>
           <t>MECCANICA COMPUTAZIONALE</t>
@@ -917,7 +909,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>CHIMICA</t>
+          <t>MATEMATICA I</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -950,11 +942,7 @@
           <t>FENOMENI DI TRASPORTO</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>RESTAURO ARCHITETTONICO</t>
-        </is>
-      </c>
+      <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="inlineStr">
         <is>
           <t>ELETTROTECNICA (I-Z)</t>
@@ -995,11 +983,7 @@
           <t>PROCESS UNIT OPERATIONS - OPERAZIONI UNITARIE NELL'INDUSTRIA DI PROCESSO</t>
         </is>
       </c>
-      <c r="AR3" t="inlineStr">
-        <is>
-          <t>COMPLEMENTI DI MATEMATICA</t>
-        </is>
-      </c>
+      <c r="AR3" t="inlineStr"/>
       <c r="AS3" t="inlineStr">
         <is>
           <t>MECCANICA COMPUTAZIONALE</t>
@@ -1107,7 +1091,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>CHIMICA</t>
+          <t>FISICA I</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -1155,22 +1139,22 @@
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr"/>
       <c r="AG4" t="inlineStr"/>
-      <c r="AH4" t="inlineStr">
+      <c r="AH4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>PROCESS PLANT OPERATIONS AND CONTROL</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr">
+        <is>
+          <t>ELETTRONICA DEI SISTEMI DIGITALI</t>
+        </is>
+      </c>
+      <c r="AK4" t="inlineStr">
         <is>
           <t>TRATTAMENTO ACQUE E RIUTILIZZO</t>
         </is>
       </c>
-      <c r="AI4" t="inlineStr">
-        <is>
-          <t>PROCESS PLANT OPERATIONS AND CONTROL</t>
-        </is>
-      </c>
-      <c r="AJ4" t="inlineStr">
-        <is>
-          <t>ELETTRONICA DEI SISTEMI DIGITALI</t>
-        </is>
-      </c>
-      <c r="AK4" t="inlineStr"/>
       <c r="AL4" t="inlineStr"/>
       <c r="AM4" t="inlineStr"/>
       <c r="AN4" t="inlineStr">
@@ -1181,11 +1165,7 @@
       <c r="AO4" t="inlineStr"/>
       <c r="AP4" t="inlineStr"/>
       <c r="AQ4" t="inlineStr"/>
-      <c r="AR4" t="inlineStr">
-        <is>
-          <t>COMPLEMENTI DI MATEMATICA</t>
-        </is>
-      </c>
+      <c r="AR4" t="inlineStr"/>
       <c r="AS4" t="inlineStr">
         <is>
           <t>MECCANICA COMPUTAZIONALE</t>
@@ -1297,7 +1277,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>FONDAMENTI DI INFORMATICA</t>
+          <t>FISICA I</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -1341,30 +1321,26 @@
         </is>
       </c>
       <c r="AC5" t="inlineStr"/>
-      <c r="AD5" t="inlineStr">
-        <is>
-          <t>LABORATORIO DI SCIENZA E TECNICA DELLE COSTRUZIONI E DI GEOTECNICA</t>
-        </is>
-      </c>
+      <c r="AD5" t="inlineStr"/>
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr"/>
       <c r="AG5" t="inlineStr"/>
-      <c r="AH5" t="inlineStr">
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>ELECTRONIC SYSTEMS FOR INDUSTRY</t>
+        </is>
+      </c>
+      <c r="AJ5" t="inlineStr">
+        <is>
+          <t>FOTOVOLTAICO E OPTOELETTRONICA</t>
+        </is>
+      </c>
+      <c r="AK5" t="inlineStr">
         <is>
           <t>TRATTAMENTO ACQUE E RIUTILIZZO</t>
         </is>
       </c>
-      <c r="AI5" t="inlineStr">
-        <is>
-          <t>ELECTRONIC SYSTEMS FOR INDUSTRY</t>
-        </is>
-      </c>
-      <c r="AJ5" t="inlineStr">
-        <is>
-          <t>FOTOVOLTAICO E OPTOELETTRONICA</t>
-        </is>
-      </c>
-      <c r="AK5" t="inlineStr"/>
       <c r="AL5" t="inlineStr"/>
       <c r="AM5" t="inlineStr"/>
       <c r="AN5" t="inlineStr">
@@ -1479,7 +1455,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>FONDAMENTI DI INFORMATICA</t>
+          <t>FISICA I</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -1511,11 +1487,7 @@
         </is>
       </c>
       <c r="AC6" t="inlineStr"/>
-      <c r="AD6" t="inlineStr">
-        <is>
-          <t>LABORATORIO DI SCIENZA E TECNICA DELLE COSTRUZIONI E DI GEOTECNICA</t>
-        </is>
-      </c>
+      <c r="AD6" t="inlineStr"/>
       <c r="AE6" t="inlineStr">
         <is>
           <t>INGLESE</t>
@@ -1523,22 +1495,22 @@
       </c>
       <c r="AF6" t="inlineStr"/>
       <c r="AG6" t="inlineStr"/>
-      <c r="AH6" t="inlineStr">
+      <c r="AH6" t="inlineStr"/>
+      <c r="AI6" t="inlineStr">
+        <is>
+          <t>ELECTRONIC SYSTEMS FOR INDUSTRY</t>
+        </is>
+      </c>
+      <c r="AJ6" t="inlineStr">
+        <is>
+          <t>FOTOVOLTAICO E OPTOELETTRONICA</t>
+        </is>
+      </c>
+      <c r="AK6" t="inlineStr">
         <is>
           <t>TRATTAMENTO ACQUE E RIUTILIZZO</t>
         </is>
       </c>
-      <c r="AI6" t="inlineStr">
-        <is>
-          <t>ELECTRONIC SYSTEMS FOR INDUSTRY</t>
-        </is>
-      </c>
-      <c r="AJ6" t="inlineStr">
-        <is>
-          <t>FOTOVOLTAICO E OPTOELETTRONICA</t>
-        </is>
-      </c>
-      <c r="AK6" t="inlineStr"/>
       <c r="AL6" t="inlineStr"/>
       <c r="AM6" t="inlineStr"/>
       <c r="AN6" t="inlineStr">
@@ -1645,7 +1617,7 @@
       <c r="S7" t="inlineStr"/>
       <c r="T7" t="inlineStr">
         <is>
-          <t>FONDAMENTI DI AUTOMATICA</t>
+          <t>FONDAMENTI DI ELETTRONICA</t>
         </is>
       </c>
       <c r="U7" t="inlineStr">
@@ -1693,7 +1665,7 @@
       </c>
       <c r="AJ7" t="inlineStr">
         <is>
-          <t>ANTENNE</t>
+          <t>MISURE E CONTROLLI PER L'AUTOMAZIONE</t>
         </is>
       </c>
       <c r="AK7" t="inlineStr"/>
@@ -1823,7 +1795,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>FONDAMENTI DI AUTOMATICA</t>
+          <t>FONDAMENTI DI ELETTRONICA</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
@@ -1877,7 +1849,7 @@
       <c r="AG8" t="inlineStr"/>
       <c r="AH8" t="inlineStr">
         <is>
-          <t>ANALISI E MITIGAZIONE DEL RISCHIO COSTIERO</t>
+          <t>COMPATIBILITA` ELETTROMAGNETICA PER APPARATI AUDIO</t>
         </is>
       </c>
       <c r="AI8" t="inlineStr">
@@ -1887,7 +1859,7 @@
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
-          <t>ANTENNE</t>
+          <t>MISURE E CONTROLLI PER L'AUTOMAZIONE</t>
         </is>
       </c>
       <c r="AK8" t="inlineStr"/>
@@ -2071,7 +2043,7 @@
       <c r="AG9" t="inlineStr"/>
       <c r="AH9" t="inlineStr">
         <is>
-          <t>ANALISI E MITIGAZIONE DEL RISCHIO COSTIERO</t>
+          <t>COMPATIBILITA` ELETTROMAGNETICA PER APPARATI AUDIO</t>
         </is>
       </c>
       <c r="AI9" t="inlineStr">
@@ -2195,7 +2167,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>FONDAMENTI DI ELETTRONICA</t>
+          <t>FONDAMENTI DI AUTOMATICA</t>
         </is>
       </c>
       <c r="U10" t="inlineStr">
@@ -2224,14 +2196,22 @@
           <t>CHIMICA INDUSTRIALE</t>
         </is>
       </c>
-      <c r="AA10" t="inlineStr"/>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>CHIMICA E TECNOLOGIA DEL RESTAURO E DELLA CONSERVAZIONE DEI MATERIALI</t>
+        </is>
+      </c>
       <c r="AB10" t="inlineStr">
         <is>
           <t>ELETTROTECNICA (A-H)</t>
         </is>
       </c>
       <c r="AC10" t="inlineStr"/>
-      <c r="AD10" t="inlineStr"/>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>LABORATORIO DI SCIENZA E TECNICA DELLE COSTRUZIONI E DI GEOTECNICA</t>
+        </is>
+      </c>
       <c r="AE10" t="inlineStr"/>
       <c r="AF10" t="inlineStr"/>
       <c r="AG10" t="inlineStr">
@@ -2239,11 +2219,7 @@
           <t>LINGUA INGLESE</t>
         </is>
       </c>
-      <c r="AH10" t="inlineStr">
-        <is>
-          <t>ANALISI E MITIGAZIONE DEL RISCHIO COSTIERO</t>
-        </is>
-      </c>
+      <c r="AH10" t="inlineStr"/>
       <c r="AI10" t="inlineStr">
         <is>
           <t>SMART POLYMERS AND ADDITIVE MANUFACTURING</t>
@@ -2251,7 +2227,7 @@
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
-          <t>MISURE E CONTROLLI PER L'AUTOMAZIONE</t>
+          <t>ANTENNE</t>
         </is>
       </c>
       <c r="AK10" t="inlineStr"/>
@@ -2273,7 +2249,11 @@
           <t>BIOCHEMICAL AND FOOD PLANT DESIGN - IMPIANTI BIOCHIMICI E DELL'INDUSTRIA ALIMENTARE_Modulo 1</t>
         </is>
       </c>
-      <c r="AR10" t="inlineStr"/>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>ELEMENTI DI GEOMORFOLOGIA</t>
+        </is>
+      </c>
       <c r="AS10" t="inlineStr">
         <is>
           <t>GESTIONE DEL TRAFFICO E MOBILITÀ SOSTENIBILE</t>
@@ -2283,7 +2263,7 @@
       <c r="AU10" t="inlineStr"/>
       <c r="AV10" t="inlineStr">
         <is>
-          <t>ELEMENTI DI GEOMORFOLOGIA</t>
+          <t>LINGUA INGLESE</t>
         </is>
       </c>
     </row>
@@ -2345,7 +2325,7 @@
       <c r="S11" t="inlineStr"/>
       <c r="T11" t="inlineStr">
         <is>
-          <t>FONDAMENTI DI ELETTRONICA</t>
+          <t>FONDAMENTI DI AUTOMATICA</t>
         </is>
       </c>
       <c r="U11" t="inlineStr">
@@ -2393,7 +2373,7 @@
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>MISURE E CONTROLLI PER L'AUTOMAZIONE</t>
+          <t>ANTENNE</t>
         </is>
       </c>
       <c r="AK11" t="inlineStr"/>
@@ -2415,13 +2395,17 @@
           <t>BIOCHEMICAL AND FOOD PLANT DESIGN - IMPIANTI BIOCHIMICI E DELL'INDUSTRIA ALIMENTARE_Modulo 1</t>
         </is>
       </c>
-      <c r="AR11" t="inlineStr"/>
+      <c r="AR11" t="inlineStr">
+        <is>
+          <t>ELEMENTI DI GEOMORFOLOGIA</t>
+        </is>
+      </c>
       <c r="AS11" t="inlineStr"/>
       <c r="AT11" t="inlineStr"/>
       <c r="AU11" t="inlineStr"/>
       <c r="AV11" t="inlineStr">
         <is>
-          <t>ELEMENTI DI GEOMORFOLOGIA</t>
+          <t>LINGUA INGLESE</t>
         </is>
       </c>
     </row>
@@ -2737,7 +2721,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>INFRASTRUTTURE IDRAULICHE</t>
+          <t>ARCHITETTURA TECNICA</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -2747,12 +2731,12 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>GENERATIVE AI</t>
+          <t>ARTIFICIAL VISION</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>ARCHITETTURA TECNICA</t>
+          <t>RESTAURO ARCHITETTONICO</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -2762,7 +2746,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>CHIMICA</t>
+          <t>MATEMATICA I</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -2827,12 +2811,12 @@
       </c>
       <c r="AO2" t="inlineStr"/>
       <c r="AP2" t="inlineStr"/>
-      <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr">
-        <is>
-          <t>COMPLEMENTI DI MATEMATICA</t>
-        </is>
-      </c>
+      <c r="AQ2" t="inlineStr">
+        <is>
+          <t>INFRASTRUTTURE IDRAULICHE</t>
+        </is>
+      </c>
+      <c r="AR2" t="inlineStr"/>
       <c r="AS2" t="inlineStr">
         <is>
           <t>SUSTAINABLE ENVIRONMENTAL ENGINEERING: FROM WASTE TO VALUE</t>
@@ -2911,7 +2895,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>INFRASTRUTTURE IDRAULICHE</t>
+          <t>ARCHITETTURA TECNICA</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
@@ -2921,12 +2905,12 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>GENERATIVE AI</t>
+          <t>ARTIFICIAL VISION</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>ARCHITETTURA TECNICA</t>
+          <t>RESTAURO ARCHITETTONICO</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -2936,29 +2920,29 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
+          <t>MATEMATICA I</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>MATEMATICA I</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>FONDAMENTI DI PROGRAMMAZIONE (I-Z)</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>DISEGNO</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
           <t>CHIMICA</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>MATEMATICA I</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>FONDAMENTI DI PROGRAMMAZIONE (I-Z)</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>DISEGNO</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>CHIMICA</t>
-        </is>
-      </c>
       <c r="Y3" t="inlineStr">
         <is>
           <t>DESIGN AND ANALYSIS OF ALGORITHMS (A-H)</t>
@@ -2980,15 +2964,15 @@
         </is>
       </c>
       <c r="AC3" t="inlineStr"/>
-      <c r="AD3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>GESTIONE, RIQUALIFICAZIONE E SICUREZZA DELLE GALLERIE STRADALI</t>
+        </is>
+      </c>
       <c r="AE3" t="inlineStr"/>
       <c r="AF3" t="inlineStr"/>
       <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr">
-        <is>
-          <t>GESTIONE, RIQUALIFICAZIONE E SICUREZZA DELLE GALLERIE STRADALI</t>
-        </is>
-      </c>
+      <c r="AH3" t="inlineStr"/>
       <c r="AI3" t="inlineStr">
         <is>
           <t>ELECTRONIC SYSTEMS FOR INDUSTRY</t>
@@ -3013,12 +2997,12 @@
         </is>
       </c>
       <c r="AP3" t="inlineStr"/>
-      <c r="AQ3" t="inlineStr"/>
-      <c r="AR3" t="inlineStr">
-        <is>
-          <t>COMPLEMENTI DI MATEMATICA</t>
-        </is>
-      </c>
+      <c r="AQ3" t="inlineStr">
+        <is>
+          <t>INFRASTRUTTURE IDRAULICHE</t>
+        </is>
+      </c>
+      <c r="AR3" t="inlineStr"/>
       <c r="AS3" t="inlineStr">
         <is>
           <t>SUSTAINABLE ENVIRONMENTAL ENGINEERING: FROM WASTE TO VALUE</t>
@@ -3099,11 +3083,7 @@
           <t>INTERNET OF THINGS</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>INFRASTRUTTURE IDRAULICHE</t>
-        </is>
-      </c>
+      <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
           <t>TECNOLOGIE INFORMATICHE PER IL MONITORAGGIO CLINICO</t>
@@ -3126,7 +3106,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>CHIMICA</t>
+          <t>FONDAMENTI DI INFORMATICA</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -3170,15 +3150,15 @@
         </is>
       </c>
       <c r="AC4" t="inlineStr"/>
-      <c r="AD4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>GESTIONE, RIQUALIFICAZIONE E SICUREZZA DELLE GALLERIE STRADALI</t>
+        </is>
+      </c>
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr"/>
       <c r="AG4" t="inlineStr"/>
-      <c r="AH4" t="inlineStr">
-        <is>
-          <t>GESTIONE, RIQUALIFICAZIONE E SICUREZZA DELLE GALLERIE STRADALI</t>
-        </is>
-      </c>
+      <c r="AH4" t="inlineStr"/>
       <c r="AI4" t="inlineStr">
         <is>
           <t>ELECTRONIC SYSTEMS FOR INDUSTRY</t>
@@ -3203,12 +3183,12 @@
         </is>
       </c>
       <c r="AP4" t="inlineStr"/>
-      <c r="AQ4" t="inlineStr"/>
-      <c r="AR4" t="inlineStr">
-        <is>
-          <t>COMPLEMENTI DI MATEMATICA</t>
-        </is>
-      </c>
+      <c r="AQ4" t="inlineStr">
+        <is>
+          <t>INFRASTRUTTURE IDRAULICHE</t>
+        </is>
+      </c>
+      <c r="AR4" t="inlineStr"/>
       <c r="AS4" t="inlineStr">
         <is>
           <t>SUSTAINABLE ENVIRONMENTAL ENGINEERING: FROM WASTE TO VALUE</t>
@@ -3301,7 +3281,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>ARTIFICIAL VISION</t>
+          <t>GENERATIVE AI</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -3356,15 +3336,15 @@
         </is>
       </c>
       <c r="AC5" t="inlineStr"/>
-      <c r="AD5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>GESTIONE, RIQUALIFICAZIONE E SICUREZZA DELLE GALLERIE STRADALI</t>
+        </is>
+      </c>
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr"/>
       <c r="AG5" t="inlineStr"/>
-      <c r="AH5" t="inlineStr">
-        <is>
-          <t>GESTIONE, RIQUALIFICAZIONE E SICUREZZA DELLE GALLERIE STRADALI</t>
-        </is>
-      </c>
+      <c r="AH5" t="inlineStr"/>
       <c r="AI5" t="inlineStr">
         <is>
           <t>COMPUTER SCIENCE FOR INDUSTRY 4.0: NETWORKING, BIG DATA MANAGEMENT AND MACHINE LEARNING</t>
@@ -3391,7 +3371,7 @@
       <c r="AP5" t="inlineStr"/>
       <c r="AQ5" t="inlineStr">
         <is>
-          <t>BIOCHEMICAL AND FOOD PLANT DESIGN - IMPIANTI BIOCHIMICI E DELL'INDUSTRIA ALIMENTARE_Modulo 2</t>
+          <t>MATHEMATICAL MODELING OF PROCESSES IN FOOD INDUSTRIES - MODELLISTICA MATEMATICA DEI PROCESSI DELL'INDUSTRIA ALIMENTARE</t>
         </is>
       </c>
       <c r="AR5" t="inlineStr">
@@ -3399,11 +3379,7 @@
           <t>PIANIFICAZIONE TERRITORIALE</t>
         </is>
       </c>
-      <c r="AS5" t="inlineStr">
-        <is>
-          <t>LABORATORIO DI SCIENZA E TECNICA DELLE COSTRUZIONI E DI GEOTECNICA</t>
-        </is>
-      </c>
+      <c r="AS5" t="inlineStr"/>
       <c r="AT5" t="inlineStr">
         <is>
           <t>AEROMOBILI A PILOTAGGIO REMOTO: BASI TEORICHE E APPLICAZIONI</t>
@@ -3491,7 +3467,7 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>ARTIFICIAL VISION</t>
+          <t>GENERATIVE AI</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -3538,7 +3514,11 @@
       </c>
       <c r="AB6" t="inlineStr"/>
       <c r="AC6" t="inlineStr"/>
-      <c r="AD6" t="inlineStr"/>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>LABORATORIO DI SCIENZA E TECNICA DELLE COSTRUZIONI E DI GEOTECNICA</t>
+        </is>
+      </c>
       <c r="AE6" t="inlineStr">
         <is>
           <t>INGLESE</t>
@@ -3573,7 +3553,7 @@
       <c r="AP6" t="inlineStr"/>
       <c r="AQ6" t="inlineStr">
         <is>
-          <t>BIOCHEMICAL AND FOOD PLANT DESIGN - IMPIANTI BIOCHIMICI E DELL'INDUSTRIA ALIMENTARE_Modulo 2</t>
+          <t>MATHEMATICAL MODELING OF PROCESSES IN FOOD INDUSTRIES - MODELLISTICA MATEMATICA DEI PROCESSI DELL'INDUSTRIA ALIMENTARE</t>
         </is>
       </c>
       <c r="AR6" t="inlineStr">
@@ -3581,11 +3561,7 @@
           <t>PIANIFICAZIONE TERRITORIALE</t>
         </is>
       </c>
-      <c r="AS6" t="inlineStr">
-        <is>
-          <t>LABORATORIO DI SCIENZA E TECNICA DELLE COSTRUZIONI E DI GEOTECNICA</t>
-        </is>
-      </c>
+      <c r="AS6" t="inlineStr"/>
       <c r="AT6" t="inlineStr">
         <is>
           <t>AEROMOBILI A PILOTAGGIO REMOTO: BASI TEORICHE E APPLICAZIONI</t>
@@ -3657,7 +3633,11 @@
           <t>5G NETWORKS</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr"/>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>URBANISTICA</t>
+        </is>
+      </c>
       <c r="P7" t="inlineStr">
         <is>
           <t>GESTIONE DELL'INNOVAZIONE E DELLA TECNOLOGIA</t>
@@ -3704,7 +3684,11 @@
       </c>
       <c r="AB7" t="inlineStr"/>
       <c r="AC7" t="inlineStr"/>
-      <c r="AD7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>LABORATORIO DI SCIENZA E TECNICA DELLE COSTRUZIONI E DI GEOTECNICA</t>
+        </is>
+      </c>
       <c r="AE7" t="inlineStr">
         <is>
           <t>INGLESE</t>
@@ -3743,11 +3727,7 @@
           <t>DESIGN OF EMBEDDED DIGITAL CONTROLLERS</t>
         </is>
       </c>
-      <c r="AS7" t="inlineStr">
-        <is>
-          <t>LABORATORIO DI SCIENZA E TECNICA DELLE COSTRUZIONI E DI GEOTECNICA</t>
-        </is>
-      </c>
+      <c r="AS7" t="inlineStr"/>
       <c r="AT7" t="inlineStr"/>
       <c r="AU7" t="inlineStr">
         <is>
@@ -3789,7 +3769,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>BIOLOGY AND GENOMICS</t>
+          <t>MEDICAL SOFTWARE ENGINEERING</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -3817,22 +3797,22 @@
       <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr">
         <is>
+          <t>URBANISTICA</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>ELABORAZIONE DI SEGNALI E DATI BIOMEDICI</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>ANALISI MATEMATICA 1</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
           <t>ANALISI DEI DATI FISICI ED ACUSTICA</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>ELABORAZIONE DI SEGNALI E DATI BIOMEDICI</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>ANALISI MATEMATICA 1</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>URBANISTICA</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -3921,7 +3901,7 @@
       <c r="AP8" t="inlineStr"/>
       <c r="AQ8" t="inlineStr">
         <is>
-          <t>MATHEMATICAL MODELING OF PROCESSES IN FOOD INDUSTRIES - MODELLISTICA MATEMATICA DEI PROCESSI DELL'INDUSTRIA ALIMENTARE</t>
+          <t>BIOCHEMICAL AND FOOD PLANT DESIGN - IMPIANTI BIOCHIMICI E DELL'INDUSTRIA ALIMENTARE_Modulo 2</t>
         </is>
       </c>
       <c r="AR8" t="inlineStr">
@@ -3964,14 +3944,10 @@
           <t>PROGETTAZIONE DI STRUTTURE SISMO-RESISTENTI E BIM</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>MODELLAZIONE DI SISTEMI PRODUTTIVI E LOGISTICI</t>
-        </is>
-      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>BIOLOGY AND GENOMICS</t>
+          <t>MEDICAL SOFTWARE ENGINEERING</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -4003,22 +3979,22 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
+          <t>URBANISTICA</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>ELABORAZIONE DI SEGNALI E DATI BIOMEDICI</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>ANALISI MATEMATICA 1</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
           <t>ANALISI DEI DATI FISICI ED ACUSTICA</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>ELABORAZIONE DI SEGNALI E DATI BIOMEDICI</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>ANALISI MATEMATICA 1</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>URBANISTICA</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -4107,7 +4083,7 @@
       <c r="AP9" t="inlineStr"/>
       <c r="AQ9" t="inlineStr">
         <is>
-          <t>MATHEMATICAL MODELING OF PROCESSES IN FOOD INDUSTRIES - MODELLISTICA MATEMATICA DEI PROCESSI DELL'INDUSTRIA ALIMENTARE</t>
+          <t>BIOCHEMICAL AND FOOD PLANT DESIGN - IMPIANTI BIOCHIMICI E DELL'INDUSTRIA ALIMENTARE_Modulo 2</t>
         </is>
       </c>
       <c r="AR9" t="inlineStr">
@@ -4150,11 +4126,7 @@
           <t>PROGETTAZIONE DI STRUTTURE SISMO-RESISTENTI E BIM</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>MODELLAZIONE DI SISTEMI PRODUTTIVI E LOGISTICI</t>
-        </is>
-      </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>HEALTH DATA ANALYTICS</t>
@@ -4187,22 +4159,22 @@
           <t>TECNOLOGIE WEB</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>ALGORITMI E STRUTTURE DATI</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>FONDAMENTI DI PROGRAMMAZIONE</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
         <is>
           <t>GEOLOGIA E GEOMORFOLOGIA</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>ALGORITMI E STRUTTURE DATI</t>
-        </is>
-      </c>
-      <c r="Q10" t="inlineStr">
-        <is>
-          <t>FONDAMENTI DI PROGRAMMAZIONE</t>
-        </is>
-      </c>
-      <c r="R10" t="inlineStr"/>
       <c r="S10" t="inlineStr">
         <is>
           <t>MODELLI E APPLICAZIONI DEL METODO DEGLI ELEMENTI FINITI DELL'INGEGNERIA CIVILE</t>
@@ -4243,11 +4215,7 @@
           <t>TERMODINAMICA DELL'INGEGNERIA CHIMICA</t>
         </is>
       </c>
-      <c r="AA10" t="inlineStr">
-        <is>
-          <t>CHIMICA E TECNOLOGIA DEL RESTAURO E DELLA CONSERVAZIONE DEI MATERIALI</t>
-        </is>
-      </c>
+      <c r="AA10" t="inlineStr"/>
       <c r="AB10" t="inlineStr">
         <is>
           <t>ANALISI DEI SEGNALI (A-H)</t>
@@ -4332,11 +4300,7 @@
           <t>PROGETTAZIONE DI STRUTTURE SISMO-RESISTENTI E BIM</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>MODELLAZIONE DI SISTEMI PRODUTTIVI E LOGISTICI</t>
-        </is>
-      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>HEALTH DATA ANALYTICS</t>
@@ -4369,22 +4333,22 @@
           <t>TECNOLOGIE WEB</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>ALGORITMI E STRUTTURE DATI</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>FONDAMENTI DI PROGRAMMAZIONE</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
         <is>
           <t>GEOLOGIA E GEOMORFOLOGIA</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>ALGORITMI E STRUTTURE DATI</t>
-        </is>
-      </c>
-      <c r="Q11" t="inlineStr">
-        <is>
-          <t>FONDAMENTI DI PROGRAMMAZIONE</t>
-        </is>
-      </c>
-      <c r="R11" t="inlineStr"/>
       <c r="S11" t="inlineStr">
         <is>
           <t>MODELLI E APPLICAZIONI DEL METODO DEGLI ELEMENTI FINITI DELL'INGEGNERIA CIVILE</t>
@@ -4770,7 +4734,7 @@
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>MARKETING E SVILUPPO PRODOTTO</t>
+          <t>ADVANCED MATHEMATICS - COMPLEMENTI DI MATEMATICA</t>
         </is>
       </c>
       <c r="J2" t="inlineStr"/>
@@ -4806,47 +4770,47 @@
           <t>ARCHITETTURA TECNICA</t>
         </is>
       </c>
-      <c r="S2" t="inlineStr">
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>FISICA I</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>MATEMATICA I</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>HIGH PERFORMANCE COMPUTING</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>DISEGNO DELL'ARCHITETTURA</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>TERMODINAMICA DELL'INGEGNERIA CHIMICA</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>DESIGN AND ANALYSIS OF ALGORITHMS (I-Z)</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>MARKETING E SVILUPPO PRODOTTO</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
         <is>
           <t>IDRAULICA E FLUIDODINAMICA AMBIENTALE</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr">
-        <is>
-          <t>CHIMICA</t>
-        </is>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>MATEMATICA I</t>
-        </is>
-      </c>
-      <c r="V2" t="inlineStr">
-        <is>
-          <t>HIGH PERFORMANCE COMPUTING</t>
-        </is>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>DISEGNO DELL'ARCHITETTURA</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>TERMODINAMICA DELL'INGEGNERIA CHIMICA</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>DESIGN AND ANALYSIS OF ALGORITHMS (I-Z)</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>ADVANCED MATHEMATICS - COMPLEMENTI DI MATEMATICA</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr"/>
       <c r="AB2" t="inlineStr">
         <is>
           <t>ELETTROTECNICA (A-H)</t>
@@ -4887,11 +4851,7 @@
       <c r="AO2" t="inlineStr"/>
       <c r="AP2" t="inlineStr"/>
       <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr">
-        <is>
-          <t>COMPLEMENTI DI MATEMATICA</t>
-        </is>
-      </c>
+      <c r="AR2" t="inlineStr"/>
       <c r="AS2" t="inlineStr">
         <is>
           <t>PIANIFICAZIONE TERRITORIALE</t>
@@ -4944,7 +4904,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>MARKETING E SVILUPPO PRODOTTO</t>
+          <t>ADVANCED MATHEMATICS - COMPLEMENTI DI MATEMATICA</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
@@ -4984,47 +4944,47 @@
           <t>ARCHITETTURA TECNICA</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>FISICA I</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>MATEMATICA I</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>HIGH PERFORMANCE COMPUTING</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>DISEGNO DELL'ARCHITETTURA</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>TERMODINAMICA DELL'INGEGNERIA CHIMICA</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>DESIGN AND ANALYSIS OF ALGORITHMS (I-Z)</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>MARKETING E SVILUPPO PRODOTTO</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
         <is>
           <t>IDRAULICA E FLUIDODINAMICA AMBIENTALE</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr">
-        <is>
-          <t>CHIMICA</t>
-        </is>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>MATEMATICA I</t>
-        </is>
-      </c>
-      <c r="V3" t="inlineStr">
-        <is>
-          <t>HIGH PERFORMANCE COMPUTING</t>
-        </is>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>DISEGNO DELL'ARCHITETTURA</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>TERMODINAMICA DELL'INGEGNERIA CHIMICA</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>DESIGN AND ANALYSIS OF ALGORITHMS (I-Z)</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>ADVANCED MATHEMATICS - COMPLEMENTI DI MATEMATICA</t>
-        </is>
-      </c>
-      <c r="AA3" t="inlineStr"/>
       <c r="AB3" t="inlineStr">
         <is>
           <t>ELETTROTECNICA (A-H)</t>
@@ -5069,11 +5029,7 @@
       <c r="AO3" t="inlineStr"/>
       <c r="AP3" t="inlineStr"/>
       <c r="AQ3" t="inlineStr"/>
-      <c r="AR3" t="inlineStr">
-        <is>
-          <t>COMPLEMENTI DI MATEMATICA</t>
-        </is>
-      </c>
+      <c r="AR3" t="inlineStr"/>
       <c r="AS3" t="inlineStr">
         <is>
           <t>PIANIFICAZIONE TERRITORIALE</t>
@@ -5122,7 +5078,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>MARKETING E SVILUPPO PRODOTTO</t>
+          <t>ADVANCED MATHEMATICS - COMPLEMENTI DI MATEMATICA</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -5173,7 +5129,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>CHIMICA</t>
+          <t>FISICA I</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -5203,7 +5159,7 @@
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>ADVANCED MATHEMATICS - COMPLEMENTI DI MATEMATICA</t>
+          <t>MARKETING E SVILUPPO PRODOTTO</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
@@ -5259,21 +5215,13 @@
           <t>REATTORI CHIMICI ALIMENTARI</t>
         </is>
       </c>
-      <c r="AR4" t="inlineStr">
-        <is>
-          <t>COMPLEMENTI DI MATEMATICA</t>
-        </is>
-      </c>
+      <c r="AR4" t="inlineStr"/>
       <c r="AS4" t="inlineStr">
         <is>
           <t>PIANIFICAZIONE TERRITORIALE</t>
         </is>
       </c>
-      <c r="AT4" t="inlineStr">
-        <is>
-          <t>AEROMOBILI A PILOTAGGIO REMOTO: BASI TEORICHE E APPLICAZIONI</t>
-        </is>
-      </c>
+      <c r="AT4" t="inlineStr"/>
       <c r="AU4" t="inlineStr"/>
       <c r="AV4" t="inlineStr"/>
     </row>
@@ -5371,7 +5319,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>FONDAMENTI DI INFORMATICA</t>
+          <t>MATEMATICA I</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -5463,11 +5411,7 @@
         </is>
       </c>
       <c r="AS5" t="inlineStr"/>
-      <c r="AT5" t="inlineStr">
-        <is>
-          <t>AEROMOBILI A PILOTAGGIO REMOTO: BASI TEORICHE E APPLICAZIONI</t>
-        </is>
-      </c>
+      <c r="AT5" t="inlineStr"/>
       <c r="AU5" t="inlineStr"/>
       <c r="AV5" t="inlineStr"/>
     </row>
@@ -5557,7 +5501,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>FONDAMENTI DI INFORMATICA</t>
+          <t>MATEMATICA I</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -5645,11 +5589,7 @@
         </is>
       </c>
       <c r="AS6" t="inlineStr"/>
-      <c r="AT6" t="inlineStr">
-        <is>
-          <t>AEROMOBILI A PILOTAGGIO REMOTO: BASI TEORICHE E APPLICAZIONI</t>
-        </is>
-      </c>
+      <c r="AT6" t="inlineStr"/>
       <c r="AU6" t="inlineStr"/>
       <c r="AV6" t="inlineStr"/>
     </row>
@@ -5706,22 +5646,22 @@
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr">
         <is>
+          <t>URBANISTICA</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>PROFESSIONAL SKILLS AND KNOWLEDGE</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>AUTONOMOUS ROBOTICS FOR LAND, SEA AND SKY MISSIONS</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
           <t>MATEMATICA I</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>PROFESSIONAL SKILLS AND KNOWLEDGE</t>
-        </is>
-      </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>AUTONOMOUS ROBOTICS FOR LAND, SEA AND SKY MISSIONS</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>URBANISTICA</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -5767,11 +5707,7 @@
       </c>
       <c r="AF7" t="inlineStr"/>
       <c r="AG7" t="inlineStr"/>
-      <c r="AH7" t="inlineStr">
-        <is>
-          <t>COMPATIBILITA` ELETTROMAGNETICA PER APPARATI AUDIO</t>
-        </is>
-      </c>
+      <c r="AH7" t="inlineStr"/>
       <c r="AI7" t="inlineStr"/>
       <c r="AJ7" t="inlineStr">
         <is>
@@ -5801,7 +5737,11 @@
       <c r="AS7" t="inlineStr"/>
       <c r="AT7" t="inlineStr"/>
       <c r="AU7" t="inlineStr"/>
-      <c r="AV7" t="inlineStr"/>
+      <c r="AV7" t="inlineStr">
+        <is>
+          <t>AEROMOBILI A PILOTAGGIO REMOTO: BASI TEORICHE E APPLICAZIONI</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -5832,7 +5772,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>MEDICAL SOFTWARE ENGINEERING</t>
+          <t>BIOLOGY AND GENOMICS</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -5868,22 +5808,22 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
+          <t>URBANISTICA</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>CALCOLATORI ELETTRONICI</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>AUTONOMOUS ROBOTICS FOR LAND, SEA AND SKY MISSIONS</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
           <t>MATEMATICA I</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>CALCOLATORI ELETTRONICI</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>AUTONOMOUS ROBOTICS FOR LAND, SEA AND SKY MISSIONS</t>
-        </is>
-      </c>
-      <c r="R8" t="inlineStr">
-        <is>
-          <t>URBANISTICA</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -5937,11 +5877,7 @@
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr"/>
       <c r="AG8" t="inlineStr"/>
-      <c r="AH8" t="inlineStr">
-        <is>
-          <t>COMPATIBILITA` ELETTROMAGNETICA PER APPARATI AUDIO</t>
-        </is>
-      </c>
+      <c r="AH8" t="inlineStr"/>
       <c r="AI8" t="inlineStr"/>
       <c r="AJ8" t="inlineStr">
         <is>
@@ -5968,18 +5904,30 @@
       <c r="AP8" t="inlineStr"/>
       <c r="AQ8" t="inlineStr">
         <is>
+          <t>WASTE WATER TREATMENT IN PROCESS INDUSTRIES - TRATTAMENTO EFFLUENTI</t>
+        </is>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>LABORATORIO DI IMPIANTI, CERTIFICAZIONE ENERGETICA E PROTEZIONE AMBIENTALE</t>
+        </is>
+      </c>
+      <c r="AS8" t="inlineStr">
+        <is>
+          <t>ANALISI E MITIGAZIONE DEL RISCHIO COSTIERO</t>
+        </is>
+      </c>
+      <c r="AT8" t="inlineStr">
+        <is>
           <t>GESTIONE E RIQUALIFICAZIONE DELLE COSTRUZIONI IDRAULICHE</t>
         </is>
       </c>
-      <c r="AR8" t="inlineStr">
-        <is>
-          <t>LABORATORIO DI IMPIANTI, CERTIFICAZIONE ENERGETICA E PROTEZIONE AMBIENTALE</t>
-        </is>
-      </c>
-      <c r="AS8" t="inlineStr"/>
-      <c r="AT8" t="inlineStr"/>
       <c r="AU8" t="inlineStr"/>
-      <c r="AV8" t="inlineStr"/>
+      <c r="AV8" t="inlineStr">
+        <is>
+          <t>AEROMOBILI A PILOTAGGIO REMOTO: BASI TEORICHE E APPLICAZIONI</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
@@ -6014,7 +5962,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>MEDICAL SOFTWARE ENGINEERING</t>
+          <t>BIOLOGY AND GENOMICS</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -6022,11 +5970,7 @@
           <t>LABORATORIO DI ELETTRONICA</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>FLUIDODINAMICA NUMERICA</t>
-        </is>
-      </c>
+      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
           <t>SCAVI E OPERE DI SOSTEGNO</t>
@@ -6048,7 +5992,11 @@
           <t>PROGRAMMAZIONE AD OGGETTI (I-Z)</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr"/>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>URBANISTICA</t>
+        </is>
+      </c>
       <c r="P9" t="inlineStr">
         <is>
           <t>CALCOLATORI ELETTRONICI</t>
@@ -6148,20 +6096,28 @@
         </is>
       </c>
       <c r="AP9" t="inlineStr"/>
-      <c r="AQ9" t="inlineStr">
+      <c r="AQ9" t="inlineStr"/>
+      <c r="AR9" t="inlineStr">
+        <is>
+          <t>LABORATORIO DI IMPIANTI, CERTIFICAZIONE ENERGETICA E PROTEZIONE AMBIENTALE</t>
+        </is>
+      </c>
+      <c r="AS9" t="inlineStr">
+        <is>
+          <t>ANALISI E MITIGAZIONE DEL RISCHIO COSTIERO</t>
+        </is>
+      </c>
+      <c r="AT9" t="inlineStr">
         <is>
           <t>GESTIONE E RIQUALIFICAZIONE DELLE COSTRUZIONI IDRAULICHE</t>
         </is>
       </c>
-      <c r="AR9" t="inlineStr">
-        <is>
-          <t>LABORATORIO DI IMPIANTI, CERTIFICAZIONE ENERGETICA E PROTEZIONE AMBIENTALE</t>
-        </is>
-      </c>
-      <c r="AS9" t="inlineStr"/>
-      <c r="AT9" t="inlineStr"/>
       <c r="AU9" t="inlineStr"/>
-      <c r="AV9" t="inlineStr"/>
+      <c r="AV9" t="inlineStr">
+        <is>
+          <t>AEROMOBILI A PILOTAGGIO REMOTO: BASI TEORICHE E APPLICAZIONI</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
@@ -6314,18 +6270,22 @@
         </is>
       </c>
       <c r="AP10" t="inlineStr"/>
-      <c r="AQ10" t="inlineStr">
+      <c r="AQ10" t="inlineStr"/>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>LABORATORIO DI IMPIANTI, CERTIFICAZIONE ENERGETICA E PROTEZIONE AMBIENTALE</t>
+        </is>
+      </c>
+      <c r="AS10" t="inlineStr">
+        <is>
+          <t>ANALISI E MITIGAZIONE DEL RISCHIO COSTIERO</t>
+        </is>
+      </c>
+      <c r="AT10" t="inlineStr">
         <is>
           <t>GESTIONE E RIQUALIFICAZIONE DELLE COSTRUZIONI IDRAULICHE</t>
         </is>
       </c>
-      <c r="AR10" t="inlineStr">
-        <is>
-          <t>LABORATORIO DI IMPIANTI, CERTIFICAZIONE ENERGETICA E PROTEZIONE AMBIENTALE</t>
-        </is>
-      </c>
-      <c r="AS10" t="inlineStr"/>
-      <c r="AT10" t="inlineStr"/>
       <c r="AU10" t="inlineStr"/>
       <c r="AV10" t="inlineStr"/>
     </row>
@@ -6362,7 +6322,11 @@
         </is>
       </c>
       <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>FLUIDODINAMICA NUMERICA</t>
+        </is>
+      </c>
       <c r="J11" t="inlineStr">
         <is>
           <t>SCAVI E OPERE DI SOSTEGNO</t>
@@ -6728,7 +6692,11 @@
           <t>08:30-09:30</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>MECCANICA DELLE TERRE</t>
+        </is>
+      </c>
       <c r="C2" t="inlineStr">
         <is>
           <t>MECCANICA DEI FLUIDI</t>
@@ -6739,11 +6707,7 @@
           <t>CATALIZZATORI NANOSTRUTTURATI PER L'ENERGIA E L'AMBIENTE</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>MECCANICA DELLE TERRE</t>
-        </is>
-      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>LABORATORIO DI CREAZIONE D'IMPRESA</t>
@@ -6766,7 +6730,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>MECCANICA COMPUTAZIONALE</t>
+          <t>ANALISI E MITIGAZIONE DEL RISCHIO DA ALLUVIONE</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
@@ -6793,7 +6757,7 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>GENERATIVE AI</t>
+          <t>ARTIFICIAL VISION</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -6808,7 +6772,7 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
-          <t>CHIMICA</t>
+          <t>MATEMATICA III</t>
         </is>
       </c>
       <c r="U2" t="inlineStr">
@@ -6848,7 +6812,11 @@
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr"/>
       <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr">
+        <is>
+          <t>COMPATIBILITA` ELETTROMAGNETICA PER APPARATI AUDIO</t>
+        </is>
+      </c>
       <c r="AI2" t="inlineStr">
         <is>
           <t>SMART POLYMERS AND ADDITIVE MANUFACTURING</t>
@@ -6866,14 +6834,10 @@
       <c r="AO2" t="inlineStr"/>
       <c r="AP2" t="inlineStr"/>
       <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr">
-        <is>
-          <t>COMPLEMENTI DI MATEMATICA</t>
-        </is>
-      </c>
+      <c r="AR2" t="inlineStr"/>
       <c r="AS2" t="inlineStr">
         <is>
-          <t>ANALISI E MITIGAZIONE DEL RISCHIO DA ALLUVIONE</t>
+          <t>MIGLIORAMENTO SISMICO DEGLI EDIFICI ESISTENTI</t>
         </is>
       </c>
       <c r="AT2" t="inlineStr"/>
@@ -6886,7 +6850,11 @@
           <t>09:30-10:30</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>MECCANICA DELLE TERRE</t>
+        </is>
+      </c>
       <c r="C3" t="inlineStr">
         <is>
           <t>MECCANICA DEI FLUIDI</t>
@@ -6897,11 +6865,7 @@
           <t>CATALIZZATORI NANOSTRUTTURATI PER L'ENERGIA E L'AMBIENTE</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>MECCANICA DELLE TERRE</t>
-        </is>
-      </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>LABORATORIO DI CREAZIONE D'IMPRESA</t>
@@ -6924,7 +6888,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>MECCANICA COMPUTAZIONALE</t>
+          <t>ANALISI E MITIGAZIONE DEL RISCHIO DA ALLUVIONE</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -6955,7 +6919,7 @@
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>GENERATIVE AI</t>
+          <t>ARTIFICIAL VISION</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -6970,7 +6934,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>CHIMICA</t>
+          <t>MATEMATICA III</t>
         </is>
       </c>
       <c r="U3" t="inlineStr">
@@ -7001,7 +6965,7 @@
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>ESTIMO</t>
+          <t>RECUPERO E CONSERVAZIONE DEGLI EDIFICI</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
@@ -7016,16 +6980,20 @@
       <c r="AG3" t="inlineStr"/>
       <c r="AH3" t="inlineStr">
         <is>
+          <t>COMPATIBILITA` ELETTROMAGNETICA PER APPARATI AUDIO</t>
+        </is>
+      </c>
+      <c r="AI3" t="inlineStr">
+        <is>
+          <t>SMART POLYMERS AND ADDITIVE MANUFACTURING</t>
+        </is>
+      </c>
+      <c r="AJ3" t="inlineStr"/>
+      <c r="AK3" t="inlineStr">
+        <is>
           <t>CONTROLLO DELL'INQUINAMENTO ATMOSFERICO</t>
         </is>
       </c>
-      <c r="AI3" t="inlineStr">
-        <is>
-          <t>SMART POLYMERS AND ADDITIVE MANUFACTURING</t>
-        </is>
-      </c>
-      <c r="AJ3" t="inlineStr"/>
-      <c r="AK3" t="inlineStr"/>
       <c r="AL3" t="inlineStr"/>
       <c r="AM3" t="inlineStr"/>
       <c r="AN3" t="inlineStr">
@@ -7036,14 +7004,10 @@
       <c r="AO3" t="inlineStr"/>
       <c r="AP3" t="inlineStr"/>
       <c r="AQ3" t="inlineStr"/>
-      <c r="AR3" t="inlineStr">
-        <is>
-          <t>COMPLEMENTI DI MATEMATICA</t>
-        </is>
-      </c>
+      <c r="AR3" t="inlineStr"/>
       <c r="AS3" t="inlineStr">
         <is>
-          <t>ANALISI E MITIGAZIONE DEL RISCHIO DA ALLUVIONE</t>
+          <t>MIGLIORAMENTO SISMICO DEGLI EDIFICI ESISTENTI</t>
         </is>
       </c>
       <c r="AT3" t="inlineStr"/>
@@ -7083,7 +7047,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>SECURE PROGRAMMING</t>
+          <t>PENETRATION TESTING AND ETHICAL HACKING</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -7129,7 +7093,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>ARTIFICIAL VISION</t>
+          <t>GENERATIVE AI</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -7144,7 +7108,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>CHIMICA</t>
+          <t>MATEMATICA III</t>
         </is>
       </c>
       <c r="U4" t="inlineStr">
@@ -7179,7 +7143,7 @@
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>ESTIMO</t>
+          <t>RECUPERO E CONSERVAZIONE DEGLI EDIFICI</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
@@ -7188,22 +7152,30 @@
         </is>
       </c>
       <c r="AC4" t="inlineStr"/>
-      <c r="AD4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>TEORIA E PROGETTO DI PONTI</t>
+        </is>
+      </c>
       <c r="AE4" t="inlineStr"/>
       <c r="AF4" t="inlineStr"/>
       <c r="AG4" t="inlineStr"/>
       <c r="AH4" t="inlineStr">
         <is>
+          <t>COMPATIBILITA` ELETTROMAGNETICA PER APPARATI AUDIO</t>
+        </is>
+      </c>
+      <c r="AI4" t="inlineStr">
+        <is>
+          <t>SMART POLYMERS AND ADDITIVE MANUFACTURING</t>
+        </is>
+      </c>
+      <c r="AJ4" t="inlineStr"/>
+      <c r="AK4" t="inlineStr">
+        <is>
           <t>CONTROLLO DELL'INQUINAMENTO ATMOSFERICO</t>
         </is>
       </c>
-      <c r="AI4" t="inlineStr">
-        <is>
-          <t>SMART POLYMERS AND ADDITIVE MANUFACTURING</t>
-        </is>
-      </c>
-      <c r="AJ4" t="inlineStr"/>
-      <c r="AK4" t="inlineStr"/>
       <c r="AL4" t="inlineStr"/>
       <c r="AM4" t="inlineStr"/>
       <c r="AN4" t="inlineStr">
@@ -7218,17 +7190,17 @@
           <t>PROCESS UNIT OPERATIONS - OPERAZIONI UNITARIE NELL'INDUSTRIA DI PROCESSO</t>
         </is>
       </c>
-      <c r="AR4" t="inlineStr">
-        <is>
-          <t>COMPLEMENTI DI MATEMATICA</t>
-        </is>
-      </c>
+      <c r="AR4" t="inlineStr"/>
       <c r="AS4" t="inlineStr">
         <is>
           <t>MIGLIORAMENTO SISMICO DEGLI EDIFICI ESISTENTI</t>
         </is>
       </c>
-      <c r="AT4" t="inlineStr"/>
+      <c r="AT4" t="inlineStr">
+        <is>
+          <t>ANALISI E MITIGAZIONE DEL RISCHIO COSTIERO</t>
+        </is>
+      </c>
       <c r="AU4" t="inlineStr"/>
       <c r="AV4" t="inlineStr"/>
     </row>
@@ -7265,27 +7237,23 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>SECURE PROGRAMMING</t>
-        </is>
-      </c>
-      <c r="H5" t="inlineStr">
+          <t>PENETRATION TESTING AND ETHICAL HACKING</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>FLUIDODINAMICA NUMERICA</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>ANALISI E MITIGAZIONE DEL RISCHIO DA FRANA</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
         <is>
           <t>GESTIONE DELL'INNOVAZIONE E DELLA TECNOLOGIA</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>FLUIDODINAMICA NUMERICA</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>ANALISI E MITIGAZIONE DEL RISCHIO DA FRANA</t>
-        </is>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>FISICA I</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -7311,7 +7279,7 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>ARTIFICIAL VISION</t>
+          <t>GENERATIVE AI</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -7326,7 +7294,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>FONDAMENTI DI INFORMATICA</t>
+          <t>FONDAMENTI DI ELETTRONICA</t>
         </is>
       </c>
       <c r="U5" t="inlineStr">
@@ -7361,7 +7329,7 @@
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t>RECUPERO E CONSERVAZIONE DEGLI EDIFICI</t>
+          <t>ESTIMO</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
@@ -7370,22 +7338,26 @@
         </is>
       </c>
       <c r="AC5" t="inlineStr"/>
-      <c r="AD5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>TEORIA E PROGETTO DI PONTI</t>
+        </is>
+      </c>
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr"/>
       <c r="AG5" t="inlineStr"/>
-      <c r="AH5" t="inlineStr">
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr">
+        <is>
+          <t>STRUCTURAL DESIGN AND MANUFACTURING OF MECHANICAL COMPONENTS</t>
+        </is>
+      </c>
+      <c r="AJ5" t="inlineStr"/>
+      <c r="AK5" t="inlineStr">
         <is>
           <t>CONTROLLO DELL'INQUINAMENTO ATMOSFERICO</t>
         </is>
       </c>
-      <c r="AI5" t="inlineStr">
-        <is>
-          <t>STRUCTURAL DESIGN AND MANUFACTURING OF MECHANICAL COMPONENTS</t>
-        </is>
-      </c>
-      <c r="AJ5" t="inlineStr"/>
-      <c r="AK5" t="inlineStr"/>
       <c r="AL5" t="inlineStr"/>
       <c r="AM5" t="inlineStr"/>
       <c r="AN5" t="inlineStr">
@@ -7403,10 +7375,14 @@
       <c r="AR5" t="inlineStr"/>
       <c r="AS5" t="inlineStr">
         <is>
-          <t>MIGLIORAMENTO SISMICO DEGLI EDIFICI ESISTENTI</t>
-        </is>
-      </c>
-      <c r="AT5" t="inlineStr"/>
+          <t>MECCANICA COMPUTAZIONALE</t>
+        </is>
+      </c>
+      <c r="AT5" t="inlineStr">
+        <is>
+          <t>ANALISI E MITIGAZIONE DEL RISCHIO COSTIERO</t>
+        </is>
+      </c>
       <c r="AU5" t="inlineStr"/>
       <c r="AV5" t="inlineStr"/>
     </row>
@@ -7439,27 +7415,23 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>PENETRATION TESTING AND ETHICAL HACKING</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
+          <t>SECURE PROGRAMMING</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>FLUIDODINAMICA NUMERICA</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>ANALISI E MITIGAZIONE DEL RISCHIO DA FRANA</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
         <is>
           <t>GESTIONE DELL'INNOVAZIONE E DELLA TECNOLOGIA</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>FLUIDODINAMICA NUMERICA</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>ANALISI E MITIGAZIONE DEL RISCHIO DA FRANA</t>
-        </is>
-      </c>
-      <c r="K6" t="inlineStr">
-        <is>
-          <t>FISICA I</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -7500,7 +7472,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>FONDAMENTI DI INFORMATICA</t>
+          <t>FONDAMENTI DI ELETTRONICA</t>
         </is>
       </c>
       <c r="U6" t="inlineStr">
@@ -7535,7 +7507,7 @@
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t>RECUPERO E CONSERVAZIONE DEGLI EDIFICI</t>
+          <t>ESTIMO</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
@@ -7589,7 +7561,7 @@
       </c>
       <c r="AS6" t="inlineStr">
         <is>
-          <t>MIGLIORAMENTO SISMICO DEGLI EDIFICI ESISTENTI</t>
+          <t>MECCANICA COMPUTAZIONALE</t>
         </is>
       </c>
       <c r="AT6" t="inlineStr"/>
@@ -7629,7 +7601,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>PENETRATION TESTING AND ETHICAL HACKING</t>
+          <t>SECURE PROGRAMMING</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -7686,10 +7658,14 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>MATEMATICA III</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr"/>
+          <t>FONDAMENTI DI INFORMATICA</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>FISICA I</t>
+        </is>
+      </c>
       <c r="V7" t="inlineStr">
         <is>
           <t>ROBOTIC SYSTEMS</t>
@@ -7860,12 +7836,12 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>MATEMATICA III</t>
+          <t>FONDAMENTI DI INFORMATICA</t>
         </is>
       </c>
       <c r="U8" t="inlineStr">
         <is>
-          <t>CHIMICA</t>
+          <t>FISICA I</t>
         </is>
       </c>
       <c r="V8" t="inlineStr">
@@ -7998,7 +7974,11 @@
           <t>VALUTAZIONE DI IMPATTO AMBIENTALE</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>MODELLAZIONE DI SISTEMI PRODUTTIVI E LOGISTICI</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr">
         <is>
           <t>HEALTH DATA ANALYTICS</t>
@@ -8058,7 +8038,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>MATEMATICA III</t>
+          <t>MATEMATICA I</t>
         </is>
       </c>
       <c r="U9" t="inlineStr">
@@ -8104,7 +8084,7 @@
       <c r="AC9" t="inlineStr"/>
       <c r="AD9" t="inlineStr">
         <is>
-          <t>TEORIA E PROGETTO DI PONTI</t>
+          <t>DESIGN OF STEEL STRUCTURES AND BIM APPLICATIONS</t>
         </is>
       </c>
       <c r="AE9" t="inlineStr"/>
@@ -8196,10 +8176,14 @@
           <t>VALUTAZIONE DI IMPATTO AMBIENTALE</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>MODELLAZIONE DI SISTEMI PRODUTTIVI E LOGISTICI</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>BIOLOGY AND GENOMICS</t>
+          <t>MEDICAL SOFTWARE ENGINEERING</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -8260,10 +8244,14 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>FONDAMENTI DI ELETTRONICA</t>
-        </is>
-      </c>
-      <c r="U10" t="inlineStr"/>
+          <t>MATEMATICA I</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>CHIMICA</t>
+        </is>
+      </c>
       <c r="V10" t="inlineStr">
         <is>
           <t>FISICA 1 (I-Z)</t>
@@ -8294,7 +8282,7 @@
       <c r="AC10" t="inlineStr"/>
       <c r="AD10" t="inlineStr">
         <is>
-          <t>TEORIA E PROGETTO DI PONTI</t>
+          <t>DESIGN OF STEEL STRUCTURES AND BIM APPLICATIONS</t>
         </is>
       </c>
       <c r="AE10" t="inlineStr"/>
@@ -8386,10 +8374,14 @@
           <t>VALUTAZIONE DI IMPATTO AMBIENTALE</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>MODELLAZIONE DI SISTEMI PRODUTTIVI E LOGISTICI</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>BIOLOGY AND GENOMICS</t>
+          <t>MEDICAL SOFTWARE ENGINEERING</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -8442,7 +8434,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>FONDAMENTI DI ELETTRONICA</t>
+          <t>MATEMATICA I</t>
         </is>
       </c>
       <c r="U11" t="inlineStr"/>
@@ -8470,11 +8462,7 @@
         </is>
       </c>
       <c r="AC11" t="inlineStr"/>
-      <c r="AD11" t="inlineStr">
-        <is>
-          <t>TEORIA E PROGETTO DI PONTI</t>
-        </is>
-      </c>
+      <c r="AD11" t="inlineStr"/>
       <c r="AE11" t="inlineStr"/>
       <c r="AF11" t="inlineStr"/>
       <c r="AG11" t="inlineStr">
@@ -9433,7 +9421,11 @@
         </is>
       </c>
       <c r="AC5" t="inlineStr"/>
-      <c r="AD5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr">
+        <is>
+          <t>TEORIA E PROGETTO DI PONTI</t>
+        </is>
+      </c>
       <c r="AE5" t="inlineStr"/>
       <c r="AF5" t="inlineStr"/>
       <c r="AG5" t="inlineStr"/>
@@ -9442,11 +9434,7 @@
           <t>SISTEMI DI INTERFACCIA PER L'AUTOMAZIONE INDUSTRIALE</t>
         </is>
       </c>
-      <c r="AI5" t="inlineStr">
-        <is>
-          <t>TEORIA E PROGETTO DI PONTI</t>
-        </is>
-      </c>
+      <c r="AI5" t="inlineStr"/>
       <c r="AJ5" t="inlineStr">
         <is>
           <t>ANTENNE</t>
@@ -9615,16 +9603,16 @@
           <t>ORIENTAMENTO AL LAVORO</t>
         </is>
       </c>
-      <c r="AD6" t="inlineStr"/>
+      <c r="AD6" t="inlineStr">
+        <is>
+          <t>TEORIA E PROGETTO DI PONTI</t>
+        </is>
+      </c>
       <c r="AE6" t="inlineStr"/>
       <c r="AF6" t="inlineStr"/>
       <c r="AG6" t="inlineStr"/>
       <c r="AH6" t="inlineStr"/>
-      <c r="AI6" t="inlineStr">
-        <is>
-          <t>TEORIA E PROGETTO DI PONTI</t>
-        </is>
-      </c>
+      <c r="AI6" t="inlineStr"/>
       <c r="AJ6" t="inlineStr">
         <is>
           <t>ANTENNE</t>
@@ -9781,15 +9769,15 @@
           <t>ORIENTAMENTO AL LAVORO</t>
         </is>
       </c>
-      <c r="AD7" t="inlineStr"/>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>TEORIA E PROGETTO DI PONTI</t>
+        </is>
+      </c>
       <c r="AE7" t="inlineStr"/>
       <c r="AF7" t="inlineStr"/>
       <c r="AG7" t="inlineStr"/>
-      <c r="AH7" t="inlineStr">
-        <is>
-          <t>COMPATIBILITA` ELETTROMAGNETICA PER APPARATI AUDIO</t>
-        </is>
-      </c>
+      <c r="AH7" t="inlineStr"/>
       <c r="AI7" t="inlineStr">
         <is>
           <t>SMART TRANSDUCERS AND MEASUREMENT</t>
@@ -9846,11 +9834,7 @@
           <t>GESTIONE DELL'INNOVAZIONE E DELLA TECNOLOGIA</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>ANALISI E MITIGAZIONE DEL RISCHIO COSTIERO</t>
-        </is>
-      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>LABORATORIO DI PROGETTAZIONE VIRTUALE</t>
@@ -9858,7 +9842,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>MEDICAL SOFTWARE ENGINEERING</t>
+          <t>BIOLOGY AND GENOMICS</t>
         </is>
       </c>
       <c r="H8" t="inlineStr"/>
@@ -9951,11 +9935,7 @@
       <c r="AE8" t="inlineStr"/>
       <c r="AF8" t="inlineStr"/>
       <c r="AG8" t="inlineStr"/>
-      <c r="AH8" t="inlineStr">
-        <is>
-          <t>COMPATIBILITA` ELETTROMAGNETICA PER APPARATI AUDIO</t>
-        </is>
-      </c>
+      <c r="AH8" t="inlineStr"/>
       <c r="AI8" t="inlineStr">
         <is>
           <t>SMART TRANSDUCERS AND MEASUREMENT</t>
@@ -10008,11 +9988,7 @@
           <t>GESTIONE DELL'INNOVAZIONE E DELLA TECNOLOGIA</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>ANALISI E MITIGAZIONE DEL RISCHIO COSTIERO</t>
-        </is>
-      </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>LABORATORIO DI PROGETTAZIONE VIRTUALE</t>
@@ -10020,7 +9996,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>MEDICAL SOFTWARE ENGINEERING</t>
+          <t>BIOLOGY AND GENOMICS</t>
         </is>
       </c>
       <c r="H9" t="inlineStr"/>
@@ -10065,7 +10041,11 @@
           <t>CHIMICA</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr"/>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>DYNAMICS, IDENTIFICATION AND CONTROL OF MECHANICAL SYSTEMS</t>
+        </is>
+      </c>
       <c r="S9" t="inlineStr">
         <is>
           <t>FISICA TECNICA E IMPIANTI TERMOTECNICI</t>
@@ -10117,11 +10097,7 @@
       <c r="AE9" t="inlineStr"/>
       <c r="AF9" t="inlineStr"/>
       <c r="AG9" t="inlineStr"/>
-      <c r="AH9" t="inlineStr">
-        <is>
-          <t>COMPATIBILITA` ELETTROMAGNETICA PER APPARATI AUDIO</t>
-        </is>
-      </c>
+      <c r="AH9" t="inlineStr"/>
       <c r="AI9" t="inlineStr">
         <is>
           <t>STRUCTURAL DESIGN AND MANUFACTURING OF MECHANICAL COMPONENTS</t>
@@ -10153,11 +10129,7 @@
         </is>
       </c>
       <c r="AS9" t="inlineStr"/>
-      <c r="AT9" t="inlineStr">
-        <is>
-          <t>DYNAMICS, IDENTIFICATION AND CONTROL OF MECHANICAL SYSTEMS</t>
-        </is>
-      </c>
+      <c r="AT9" t="inlineStr"/>
       <c r="AU9" t="inlineStr"/>
       <c r="AV9" t="inlineStr"/>
     </row>
@@ -10215,7 +10187,11 @@
           <t>FONDAMENTI DI PROGRAMMAZIONE</t>
         </is>
       </c>
-      <c r="R10" t="inlineStr"/>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>DYNAMICS, IDENTIFICATION AND CONTROL OF MECHANICAL SYSTEMS</t>
+        </is>
+      </c>
       <c r="S10" t="inlineStr">
         <is>
           <t>FISICA TECNICA E IMPIANTI TERMOTECNICI</t>
@@ -10295,11 +10271,7 @@
         </is>
       </c>
       <c r="AS10" t="inlineStr"/>
-      <c r="AT10" t="inlineStr">
-        <is>
-          <t>DYNAMICS, IDENTIFICATION AND CONTROL OF MECHANICAL SYSTEMS</t>
-        </is>
-      </c>
+      <c r="AT10" t="inlineStr"/>
       <c r="AU10" t="inlineStr"/>
       <c r="AV10" t="inlineStr"/>
     </row>
@@ -10357,7 +10329,11 @@
           <t>FONDAMENTI DI PROGRAMMAZIONE</t>
         </is>
       </c>
-      <c r="R11" t="inlineStr"/>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>DYNAMICS, IDENTIFICATION AND CONTROL OF MECHANICAL SYSTEMS</t>
+        </is>
+      </c>
       <c r="S11" t="inlineStr">
         <is>
           <t>FISICA TECNICA E IMPIANTI TERMOTECNICI</t>
@@ -10421,11 +10397,7 @@
         </is>
       </c>
       <c r="AS11" t="inlineStr"/>
-      <c r="AT11" t="inlineStr">
-        <is>
-          <t>DYNAMICS, IDENTIFICATION AND CONTROL OF MECHANICAL SYSTEMS</t>
-        </is>
-      </c>
+      <c r="AT11" t="inlineStr"/>
       <c r="AU11" t="inlineStr"/>
       <c r="AV11" t="inlineStr"/>
     </row>

</xml_diff>